<commit_message>
Lista de pendências de EAN com o motivo de cada uma
A lista de produtos ativos sem código não dizia o que fazer com cada
linha, e as providências são bem diferentes: cadastro pai pede separar as
variações, código inventado no ERP pede gerar EAN interno, e só o que não
existe em planilha nenhuma pede ir bipar na loja.

Avisa também quando o mesmo palpite serve para várias variações — o
fornecedor usa um código só para a família e o catálogo só deixa um
cadastro ficar com ele.

O diagnóstico sai de dentro do caca-ean para lib/similar, para a busca e a
lista de pendências contarem a mesma história.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FgnKDHH1zCVziRJTDyp9tv
</commit_message>
<xml_diff>
--- a/catalogo-produtos/importador/caca-ean.xlsx
+++ b/catalogo-produtos/importador/caca-ean.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="844" uniqueCount="580">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="674" uniqueCount="460">
   <si>
     <t>Confiança</t>
   </si>
@@ -1217,366 +1217,6 @@
   </si>
   <si>
     <t>Já pertence a</t>
-  </si>
-  <si>
-    <t>Premier Raças Específicas Maltês Filhotes</t>
-  </si>
-  <si>
-    <t>7897348204473</t>
-  </si>
-  <si>
-    <t>Ração Premier Pet Raças Específicas Maltês Filhotes 2,5KG</t>
-  </si>
-  <si>
-    <t>08c56a9b-4ee1-4612-91af-1b46517835c6</t>
-  </si>
-  <si>
-    <t>MORDEDOR SORVETINHO</t>
-  </si>
-  <si>
-    <t>7893032404808</t>
-  </si>
-  <si>
-    <t>MORDEDOR SORVETINHO - Azul - 1 Unidade</t>
-  </si>
-  <si>
-    <t>0c607ef4-992c-434c-be1a-7d2433ebec43</t>
-  </si>
-  <si>
-    <t>Brinquedo Bola Interativa Porta Petisco para Cães - 13 CM - Rosa</t>
-  </si>
-  <si>
-    <t>7908364101278</t>
-  </si>
-  <si>
-    <t>Brinquedo Bola Interativa Porta Petisco para Cães - 13 CM - Azul</t>
-  </si>
-  <si>
-    <t>283ae554-53e6-4e1a-b723-4ffa3e68be8a</t>
-  </si>
-  <si>
-    <t>Ração Premier Nutrição Clínica Renal Porte Pequeno</t>
-  </si>
-  <si>
-    <t>7897348208198</t>
-  </si>
-  <si>
-    <t>Ração Premier Nutrição Clínica Renal para Cães Adultos Porte Pequeno 10Kg</t>
-  </si>
-  <si>
-    <t>2a2fb984-91b2-413d-bc12-fe15cc6e29ba</t>
-  </si>
-  <si>
-    <t>Brinquedo Bola Interativa Porta Petisco para Cães - 13 CM</t>
-  </si>
-  <si>
-    <t>310a3803-bf0e-4763-87ca-4852f4d2759a</t>
-  </si>
-  <si>
-    <t>Sementes de Frutas Feltrin – 15 Variedades à Escolha</t>
-  </si>
-  <si>
-    <t>7896061731945</t>
-  </si>
-  <si>
-    <t>Sementes de Frutas Feltrin – 15 Variedades à Escolha | Alta Qualidade e Fácil Cultivo - Fisális Goldenberry</t>
-  </si>
-  <si>
-    <t>Sementes de Frutas Feltrin – 15 Variedades à Escolha | Alta Qualidade e Fácil Cultivo - Tomate Bartô</t>
-  </si>
-  <si>
-    <t>4372113d-d268-48ff-b687-99e46ba00508</t>
-  </si>
-  <si>
-    <t>PELUCIA OSSO</t>
-  </si>
-  <si>
-    <t>7898701924717</t>
-  </si>
-  <si>
-    <t>PELUCIA OSSO - Osso</t>
-  </si>
-  <si>
-    <t>4479c1e5-715f-4e44-a1b4-a05a5d8402e1</t>
-  </si>
-  <si>
-    <t>Codigo/Referencia: C12041 - Escova rasqueadeira de botao de plastico curva  (120)</t>
-  </si>
-  <si>
-    <t>7890010120415</t>
-  </si>
-  <si>
-    <t>Escova Rasqueadeira de Botão de Plástico Curva</t>
-  </si>
-  <si>
-    <t>4defab17-0315-45af-aa2a-5e5562a9fa10</t>
-  </si>
-  <si>
-    <t>Premier Nutrição Clínica Cães Gastrointestinal Pequeno Porte</t>
-  </si>
-  <si>
-    <t>7897348207313</t>
-  </si>
-  <si>
-    <t>Ração Premier Nutrição Clínica Gastrointestinal para Cães Adultos Pequeno Porte 10,1kg</t>
-  </si>
-  <si>
-    <t>500ac644-47f8-4983-94c5-51fcda27206f</t>
-  </si>
-  <si>
-    <t>52a43a54-e11b-41b3-9b82-85d4f195a24e</t>
-  </si>
-  <si>
-    <t>Premier Nutrição Clínica Cães Gastrointestinal Pequeno Porte - 2kg</t>
-  </si>
-  <si>
-    <t>7897348207283</t>
-  </si>
-  <si>
-    <t>Ração Premier Nutrição Clínica Gastrointestinal para Cães Adultos Pequeno Porte 2kg</t>
-  </si>
-  <si>
-    <t>55c01d3a-282f-456c-b2b8-3f315c80c26e</t>
-  </si>
-  <si>
-    <t>Brinquedo de Pelúcia com Corda</t>
-  </si>
-  <si>
-    <t>7980000000017</t>
-  </si>
-  <si>
-    <t>Brinquedo de Pelúcia com Corda - Rosa</t>
-  </si>
-  <si>
-    <t>5c03b4e3-af86-4dac-b96d-41f3413a6d4b</t>
-  </si>
-  <si>
-    <t>SILICA GROSSA GREAT PETS 1,6KG</t>
-  </si>
-  <si>
-    <t>7898961193168</t>
-  </si>
-  <si>
-    <t>AREIA SILICA GROSSA 1,6KG</t>
-  </si>
-  <si>
-    <t>5e4a4885-d425-46b7-8074-210710c9c9f4</t>
-  </si>
-  <si>
-    <t>Ração Premier Nutrição Clínica Renal Porte Pequeno - 2Kg</t>
-  </si>
-  <si>
-    <t>7897348208181</t>
-  </si>
-  <si>
-    <t>Ração Premier Nutrição Clínica Renal para Cães Adultos Porte Pequeno 2Kg</t>
-  </si>
-  <si>
-    <t>61f44f80-df86-43b9-8d89-ce2c9e676400</t>
-  </si>
-  <si>
-    <t>6c8be523-5a71-48ad-a0a6-7ba37e9b7117</t>
-  </si>
-  <si>
-    <t>MORDEDOR SUPER BOWL LED</t>
-  </si>
-  <si>
-    <t>7893031903074</t>
-  </si>
-  <si>
-    <t>MORDEDOR SUPER BOWL LED - Rosa</t>
-  </si>
-  <si>
-    <t>754ae7c1-5eac-4617-b569-800ce5ffab13</t>
-  </si>
-  <si>
-    <t>Ração Farmina N&amp;D Ancestral Grain Frango e Romã Gatos Adultos Castrados 7,5kg</t>
-  </si>
-  <si>
-    <t>7898604432906</t>
-  </si>
-  <si>
-    <t>Ração Farmina N&amp;D Ancestral Grain Frango Gatos Adultos Castrados 7,5kg</t>
-  </si>
-  <si>
-    <t>784edcdd-077b-40dd-bf5f-d6a11bb96755</t>
-  </si>
-  <si>
-    <t>AREIA BIODEGRADAVEL FINA 3,8KG</t>
-  </si>
-  <si>
-    <t>7898708041691</t>
-  </si>
-  <si>
-    <t>AREIA BIODEGRADAVEL FINA - 3,8KG</t>
-  </si>
-  <si>
-    <t>81c3ae11-51f6-4206-b328-e0e6607bb38a</t>
-  </si>
-  <si>
-    <t>PEITORAL H +GUIA TOH</t>
-  </si>
-  <si>
-    <t>7908275612948</t>
-  </si>
-  <si>
-    <t>PEITORAL H +GUIA TOH - Azul - P</t>
-  </si>
-  <si>
-    <t>962028dd-5ab6-4b88-bada-b4659cc70b35</t>
-  </si>
-  <si>
-    <t>GUIA+PEITORAL DEGRADE PP</t>
-  </si>
-  <si>
-    <t>7899246013027</t>
-  </si>
-  <si>
-    <t>GUIA+PEITORAL DEGRADE PP  - Azul e Rosa</t>
-  </si>
-  <si>
-    <t>9bca8279-7760-446d-b488-43b7f8948488</t>
-  </si>
-  <si>
-    <t>COLEIRA CABRESTO</t>
-  </si>
-  <si>
-    <t>7908275613280</t>
-  </si>
-  <si>
-    <t>COLEIRA CABRESTO - Azul - M</t>
-  </si>
-  <si>
-    <t>a7e0055e-3f1a-429e-bb54-8a84c2253975</t>
-  </si>
-  <si>
-    <t>Premier Raças Específicas Maltês Filhotes - 1kg</t>
-  </si>
-  <si>
-    <t>7897348203308</t>
-  </si>
-  <si>
-    <t>Ração Premier Pet Raças Específicas Maltês Filhotes 1kg</t>
-  </si>
-  <si>
-    <t>b191be89-287d-435c-9e27-5dff08753171</t>
-  </si>
-  <si>
-    <t>Referencia/Codigo: C12111 - Escova Rasqueadeira Dispenser pelos (120)</t>
-  </si>
-  <si>
-    <t>7890010121115</t>
-  </si>
-  <si>
-    <t>Escova Rasqueadeira Dispenser pelos</t>
-  </si>
-  <si>
-    <t>bd0576a5-6ae8-483b-9407-2e9e0b96cecf</t>
-  </si>
-  <si>
-    <t>FeliComfort - Feliway Redução/Prevenção de Problemas Comportamentais de Gatos - Difusor</t>
-  </si>
-  <si>
-    <t>7896112407843</t>
-  </si>
-  <si>
-    <t>Refil FeliComfort Feliway Alívio de Estresse para Gatos - 48ml</t>
-  </si>
-  <si>
-    <t>FeliComfort - Feliway Redução/Prevenção de Problemas Comportamentais de Gatos - Difusor - Refil 48ml</t>
-  </si>
-  <si>
-    <t>c2f725f0-c43a-477e-8a8c-6060f67a001e</t>
-  </si>
-  <si>
-    <t>Zelotril 12 comprimidos para Cães e Gatos</t>
-  </si>
-  <si>
-    <t>7896006200079</t>
-  </si>
-  <si>
-    <t>Zelotril 12 comprimidos para Cães e Gatos - 50mg</t>
-  </si>
-  <si>
-    <t>c43408e9-d463-46c0-9d42-a0bdc137ebc2</t>
-  </si>
-  <si>
-    <t>Petpril 30 Comprimidos Agener União Vasodilatador - 05 mg</t>
-  </si>
-  <si>
-    <t>7896006207740</t>
-  </si>
-  <si>
-    <t>Petpril 5mg 30 comprimidos</t>
-  </si>
-  <si>
-    <t>c69ce949-b00f-490f-a63c-54f66fb8c8eb</t>
-  </si>
-  <si>
-    <t>Brinquedo Bola Interativa Porta Petisco para Cães - 13 CM - Vermelho</t>
-  </si>
-  <si>
-    <t>ce819887-8ce0-4bd2-9682-442c4ab4dd3e</t>
-  </si>
-  <si>
-    <t>d7d28855-17ab-4735-916f-b6b41aad8e1d</t>
-  </si>
-  <si>
-    <t>AREIA BIODEGRADAVEL GROSSA 3,8kg</t>
-  </si>
-  <si>
-    <t>7898708041684</t>
-  </si>
-  <si>
-    <t>AREIA BIODEGRADAVEL GROSSA - 3,8KG</t>
-  </si>
-  <si>
-    <t>e116aef0-dd5b-4a4d-b5ea-7614844307bb</t>
-  </si>
-  <si>
-    <t>Premier Nutrição Clínica Cães Hipoalergênico Proteína Hidrolisada e Mandioca Pequeno Porte</t>
-  </si>
-  <si>
-    <t>7897348207320</t>
-  </si>
-  <si>
-    <t>Ração Premier Nutrição Clínica Hipoalergênico Proteína Hidrolisada para Cães Adultos Pequeno Port 10,1kg</t>
-  </si>
-  <si>
-    <t>e2bd6434-2941-4c55-8e54-7dd0f7d6202e</t>
-  </si>
-  <si>
-    <t>e7cf1774-6ae3-4def-a9d9-87cf182988b1</t>
-  </si>
-  <si>
-    <t>COLEIRA GATO SORTIDA TOH</t>
-  </si>
-  <si>
-    <t>7436861546198</t>
-  </si>
-  <si>
-    <t>COLEIRA GATO SORTIDA TOH - Azul</t>
-  </si>
-  <si>
-    <t>f53cb870-a750-48dd-a7ab-ed3c1417ac85</t>
-  </si>
-  <si>
-    <t>COLEIRA CABRESTO - Azul - G</t>
-  </si>
-  <si>
-    <t>f928a718-77e4-458a-81fd-b61aa0441b11</t>
-  </si>
-  <si>
-    <t>Premier Nutrição Clínica Cães Cardio Porte Pequeno</t>
-  </si>
-  <si>
-    <t>7897348208136</t>
-  </si>
-  <si>
-    <t>PREMIER NUTRIÇÃO CLINICA CÃES CARDIO PEQUENO PORTE 10,1 KG</t>
-  </si>
-  <si>
-    <t>fb67659b-6b66-4f7a-abda-771d3fb7f5f8</t>
   </si>
   <si>
     <t>Marca</t>
@@ -4258,7 +3898,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="50" customWidth="1"/>
@@ -4282,584 +3922,6 @@
       </c>
       <c r="E1" s="1" t="s">
         <v>7</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>401</v>
-      </c>
-      <c r="B2" s="3" t="s">
-        <v>402</v>
-      </c>
-      <c r="C2" t="s">
-        <v>403</v>
-      </c>
-      <c r="D2" t="s">
-        <v>401</v>
-      </c>
-      <c r="E2" t="s">
-        <v>404</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>405</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>406</v>
-      </c>
-      <c r="C3" t="s">
-        <v>407</v>
-      </c>
-      <c r="D3" t="s">
-        <v>405</v>
-      </c>
-      <c r="E3" t="s">
-        <v>408</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>409</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>410</v>
-      </c>
-      <c r="C4" t="s">
-        <v>411</v>
-      </c>
-      <c r="D4" t="s">
-        <v>411</v>
-      </c>
-      <c r="E4" t="s">
-        <v>412</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>413</v>
-      </c>
-      <c r="B5" s="3" t="s">
-        <v>414</v>
-      </c>
-      <c r="C5" t="s">
-        <v>415</v>
-      </c>
-      <c r="D5" t="s">
-        <v>413</v>
-      </c>
-      <c r="E5" t="s">
-        <v>416</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>417</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>410</v>
-      </c>
-      <c r="C6" t="s">
-        <v>411</v>
-      </c>
-      <c r="D6" t="s">
-        <v>411</v>
-      </c>
-      <c r="E6" t="s">
-        <v>418</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>419</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>420</v>
-      </c>
-      <c r="C7" t="s">
-        <v>421</v>
-      </c>
-      <c r="D7" t="s">
-        <v>422</v>
-      </c>
-      <c r="E7" t="s">
-        <v>423</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>424</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>425</v>
-      </c>
-      <c r="C8" t="s">
-        <v>426</v>
-      </c>
-      <c r="D8" t="s">
-        <v>426</v>
-      </c>
-      <c r="E8" t="s">
-        <v>427</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>428</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>429</v>
-      </c>
-      <c r="C9" t="s">
-        <v>430</v>
-      </c>
-      <c r="D9" t="s">
-        <v>430</v>
-      </c>
-      <c r="E9" t="s">
-        <v>431</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>432</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>433</v>
-      </c>
-      <c r="C10" t="s">
-        <v>434</v>
-      </c>
-      <c r="D10" t="s">
-        <v>432</v>
-      </c>
-      <c r="E10" t="s">
-        <v>435</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>413</v>
-      </c>
-      <c r="B11" s="3" t="s">
-        <v>414</v>
-      </c>
-      <c r="C11" t="s">
-        <v>415</v>
-      </c>
-      <c r="D11" t="s">
-        <v>413</v>
-      </c>
-      <c r="E11" t="s">
-        <v>436</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>437</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>438</v>
-      </c>
-      <c r="C12" t="s">
-        <v>439</v>
-      </c>
-      <c r="D12" t="s">
-        <v>437</v>
-      </c>
-      <c r="E12" t="s">
-        <v>440</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>441</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>442</v>
-      </c>
-      <c r="C13" t="s">
-        <v>443</v>
-      </c>
-      <c r="D13" t="s">
-        <v>443</v>
-      </c>
-      <c r="E13" t="s">
-        <v>444</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>445</v>
-      </c>
-      <c r="B14" s="3" t="s">
-        <v>446</v>
-      </c>
-      <c r="C14" t="s">
-        <v>447</v>
-      </c>
-      <c r="D14" t="s">
-        <v>447</v>
-      </c>
-      <c r="E14" t="s">
-        <v>448</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>449</v>
-      </c>
-      <c r="B15" s="3" t="s">
-        <v>450</v>
-      </c>
-      <c r="C15" t="s">
-        <v>451</v>
-      </c>
-      <c r="D15" t="s">
-        <v>449</v>
-      </c>
-      <c r="E15" t="s">
-        <v>452</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>401</v>
-      </c>
-      <c r="B16" s="3" t="s">
-        <v>402</v>
-      </c>
-      <c r="C16" t="s">
-        <v>403</v>
-      </c>
-      <c r="D16" t="s">
-        <v>401</v>
-      </c>
-      <c r="E16" t="s">
-        <v>453</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>454</v>
-      </c>
-      <c r="B17" s="3" t="s">
-        <v>455</v>
-      </c>
-      <c r="C17" t="s">
-        <v>456</v>
-      </c>
-      <c r="D17" t="s">
-        <v>456</v>
-      </c>
-      <c r="E17" t="s">
-        <v>457</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>458</v>
-      </c>
-      <c r="B18" s="3" t="s">
-        <v>459</v>
-      </c>
-      <c r="C18" t="s">
-        <v>460</v>
-      </c>
-      <c r="D18" t="s">
-        <v>458</v>
-      </c>
-      <c r="E18" t="s">
-        <v>461</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>462</v>
-      </c>
-      <c r="B19" s="3" t="s">
-        <v>463</v>
-      </c>
-      <c r="C19" t="s">
-        <v>464</v>
-      </c>
-      <c r="D19" t="s">
-        <v>464</v>
-      </c>
-      <c r="E19" t="s">
-        <v>465</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>466</v>
-      </c>
-      <c r="B20" s="3" t="s">
-        <v>467</v>
-      </c>
-      <c r="C20" t="s">
-        <v>468</v>
-      </c>
-      <c r="D20" t="s">
-        <v>468</v>
-      </c>
-      <c r="E20" t="s">
-        <v>469</v>
-      </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>470</v>
-      </c>
-      <c r="B21" s="3" t="s">
-        <v>471</v>
-      </c>
-      <c r="C21" t="s">
-        <v>472</v>
-      </c>
-      <c r="D21" t="s">
-        <v>472</v>
-      </c>
-      <c r="E21" t="s">
-        <v>473</v>
-      </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>474</v>
-      </c>
-      <c r="B22" s="3" t="s">
-        <v>475</v>
-      </c>
-      <c r="C22" t="s">
-        <v>476</v>
-      </c>
-      <c r="D22" t="s">
-        <v>476</v>
-      </c>
-      <c r="E22" t="s">
-        <v>477</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>478</v>
-      </c>
-      <c r="B23" s="3" t="s">
-        <v>479</v>
-      </c>
-      <c r="C23" t="s">
-        <v>480</v>
-      </c>
-      <c r="D23" t="s">
-        <v>478</v>
-      </c>
-      <c r="E23" t="s">
-        <v>481</v>
-      </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>482</v>
-      </c>
-      <c r="B24" s="3" t="s">
-        <v>483</v>
-      </c>
-      <c r="C24" t="s">
-        <v>484</v>
-      </c>
-      <c r="D24" t="s">
-        <v>484</v>
-      </c>
-      <c r="E24" t="s">
-        <v>485</v>
-      </c>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>486</v>
-      </c>
-      <c r="B25" s="3" t="s">
-        <v>487</v>
-      </c>
-      <c r="C25" t="s">
-        <v>488</v>
-      </c>
-      <c r="D25" t="s">
-        <v>489</v>
-      </c>
-      <c r="E25" t="s">
-        <v>490</v>
-      </c>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>491</v>
-      </c>
-      <c r="B26" s="3" t="s">
-        <v>492</v>
-      </c>
-      <c r="C26" t="s">
-        <v>493</v>
-      </c>
-      <c r="D26" t="s">
-        <v>493</v>
-      </c>
-      <c r="E26" t="s">
-        <v>494</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>495</v>
-      </c>
-      <c r="B27" s="3" t="s">
-        <v>496</v>
-      </c>
-      <c r="C27" t="s">
-        <v>497</v>
-      </c>
-      <c r="D27" t="s">
-        <v>495</v>
-      </c>
-      <c r="E27" t="s">
-        <v>498</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>499</v>
-      </c>
-      <c r="B28" s="3" t="s">
-        <v>410</v>
-      </c>
-      <c r="C28" t="s">
-        <v>411</v>
-      </c>
-      <c r="D28" t="s">
-        <v>411</v>
-      </c>
-      <c r="E28" t="s">
-        <v>500</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>432</v>
-      </c>
-      <c r="B29" s="3" t="s">
-        <v>433</v>
-      </c>
-      <c r="C29" t="s">
-        <v>434</v>
-      </c>
-      <c r="D29" t="s">
-        <v>432</v>
-      </c>
-      <c r="E29" t="s">
-        <v>501</v>
-      </c>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>502</v>
-      </c>
-      <c r="B30" s="3" t="s">
-        <v>503</v>
-      </c>
-      <c r="C30" t="s">
-        <v>504</v>
-      </c>
-      <c r="D30" t="s">
-        <v>504</v>
-      </c>
-      <c r="E30" t="s">
-        <v>505</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>506</v>
-      </c>
-      <c r="B31" s="3" t="s">
-        <v>507</v>
-      </c>
-      <c r="C31" t="s">
-        <v>508</v>
-      </c>
-      <c r="D31" t="s">
-        <v>506</v>
-      </c>
-      <c r="E31" t="s">
-        <v>509</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>506</v>
-      </c>
-      <c r="B32" s="3" t="s">
-        <v>507</v>
-      </c>
-      <c r="C32" t="s">
-        <v>508</v>
-      </c>
-      <c r="D32" t="s">
-        <v>506</v>
-      </c>
-      <c r="E32" t="s">
-        <v>510</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>511</v>
-      </c>
-      <c r="B33" s="3" t="s">
-        <v>512</v>
-      </c>
-      <c r="C33" t="s">
-        <v>513</v>
-      </c>
-      <c r="D33" t="s">
-        <v>513</v>
-      </c>
-      <c r="E33" t="s">
-        <v>514</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>515</v>
-      </c>
-      <c r="B34" s="3" t="s">
-        <v>475</v>
-      </c>
-      <c r="C34" t="s">
-        <v>476</v>
-      </c>
-      <c r="D34" t="s">
-        <v>476</v>
-      </c>
-      <c r="E34" t="s">
-        <v>516</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>517</v>
-      </c>
-      <c r="B35" s="3" t="s">
-        <v>518</v>
-      </c>
-      <c r="C35" t="s">
-        <v>519</v>
-      </c>
-      <c r="D35" t="s">
-        <v>519</v>
-      </c>
-      <c r="E35" t="s">
-        <v>520</v>
       </c>
     </row>
   </sheetData>
@@ -4884,10 +3946,10 @@
         <v>1</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>521</v>
+        <v>401</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>522</v>
+        <v>402</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>7</v>
@@ -4895,119 +3957,119 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>523</v>
+        <v>403</v>
       </c>
       <c r="B2" t="s">
-        <v>524</v>
+        <v>404</v>
       </c>
       <c r="C2" t="s">
         <v>13</v>
       </c>
       <c r="D2" t="s">
-        <v>525</v>
+        <v>405</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>526</v>
+        <v>406</v>
       </c>
       <c r="B3" t="s">
-        <v>527</v>
+        <v>407</v>
       </c>
       <c r="C3" t="s">
         <v>13</v>
       </c>
       <c r="D3" t="s">
-        <v>528</v>
+        <v>408</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>529</v>
+        <v>409</v>
       </c>
       <c r="B4" t="s">
-        <v>530</v>
+        <v>410</v>
       </c>
       <c r="C4" t="s">
         <v>13</v>
       </c>
       <c r="D4" t="s">
-        <v>531</v>
+        <v>411</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>532</v>
+        <v>412</v>
       </c>
       <c r="B5" t="s">
-        <v>533</v>
+        <v>413</v>
       </c>
       <c r="C5" t="s">
         <v>13</v>
       </c>
       <c r="D5" t="s">
-        <v>534</v>
+        <v>414</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>535</v>
+        <v>415</v>
       </c>
       <c r="B6" t="s">
-        <v>524</v>
+        <v>404</v>
       </c>
       <c r="C6" t="s">
         <v>13</v>
       </c>
       <c r="D6" t="s">
-        <v>536</v>
+        <v>416</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>537</v>
+        <v>417</v>
       </c>
       <c r="B7" t="s">
-        <v>538</v>
+        <v>418</v>
       </c>
       <c r="C7" t="s">
         <v>13</v>
       </c>
       <c r="D7" t="s">
-        <v>539</v>
+        <v>419</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>540</v>
+        <v>420</v>
       </c>
       <c r="B8" t="s">
-        <v>524</v>
+        <v>404</v>
       </c>
       <c r="C8" t="s">
         <v>13</v>
       </c>
       <c r="D8" t="s">
-        <v>541</v>
+        <v>421</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>542</v>
+        <v>422</v>
       </c>
       <c r="B9" t="s">
-        <v>530</v>
+        <v>410</v>
       </c>
       <c r="C9" t="s">
         <v>13</v>
       </c>
       <c r="D9" t="s">
-        <v>543</v>
+        <v>423</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>544</v>
+        <v>424</v>
       </c>
       <c r="B10" t="s">
         <v>13</v>
@@ -5016,180 +4078,180 @@
         <v>13</v>
       </c>
       <c r="D10" t="s">
-        <v>545</v>
+        <v>425</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>546</v>
+        <v>426</v>
       </c>
       <c r="B11" t="s">
-        <v>524</v>
+        <v>404</v>
       </c>
       <c r="C11" t="s">
-        <v>547</v>
+        <v>427</v>
       </c>
       <c r="D11" t="s">
-        <v>548</v>
+        <v>428</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>549</v>
+        <v>429</v>
       </c>
       <c r="B12" t="s">
-        <v>533</v>
+        <v>413</v>
       </c>
       <c r="C12" t="s">
         <v>13</v>
       </c>
       <c r="D12" t="s">
-        <v>550</v>
+        <v>430</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>551</v>
+        <v>431</v>
       </c>
       <c r="B13" t="s">
-        <v>524</v>
+        <v>404</v>
       </c>
       <c r="C13" t="s">
         <v>13</v>
       </c>
       <c r="D13" t="s">
-        <v>552</v>
+        <v>432</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>553</v>
+        <v>433</v>
       </c>
       <c r="B14" t="s">
-        <v>530</v>
+        <v>410</v>
       </c>
       <c r="C14" t="s">
         <v>13</v>
       </c>
       <c r="D14" t="s">
-        <v>554</v>
+        <v>434</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>555</v>
+        <v>435</v>
       </c>
       <c r="B15" t="s">
-        <v>524</v>
+        <v>404</v>
       </c>
       <c r="C15" t="s">
         <v>13</v>
       </c>
       <c r="D15" t="s">
-        <v>556</v>
+        <v>436</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>557</v>
+        <v>437</v>
       </c>
       <c r="B16" t="s">
-        <v>524</v>
+        <v>404</v>
       </c>
       <c r="C16" t="s">
         <v>13</v>
       </c>
       <c r="D16" t="s">
-        <v>558</v>
+        <v>438</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>559</v>
+        <v>439</v>
       </c>
       <c r="B17" t="s">
-        <v>524</v>
+        <v>404</v>
       </c>
       <c r="C17" t="s">
         <v>13</v>
       </c>
       <c r="D17" t="s">
-        <v>560</v>
+        <v>440</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>561</v>
+        <v>441</v>
       </c>
       <c r="B18" t="s">
-        <v>530</v>
+        <v>410</v>
       </c>
       <c r="C18" t="s">
         <v>13</v>
       </c>
       <c r="D18" t="s">
-        <v>562</v>
+        <v>442</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>563</v>
+        <v>443</v>
       </c>
       <c r="B19" t="s">
-        <v>530</v>
+        <v>410</v>
       </c>
       <c r="C19" t="s">
-        <v>564</v>
+        <v>444</v>
       </c>
       <c r="D19" t="s">
-        <v>565</v>
+        <v>445</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>566</v>
+        <v>446</v>
       </c>
       <c r="B20" t="s">
-        <v>533</v>
+        <v>413</v>
       </c>
       <c r="C20" t="s">
         <v>13</v>
       </c>
       <c r="D20" t="s">
-        <v>567</v>
+        <v>447</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>568</v>
+        <v>448</v>
       </c>
       <c r="B21" t="s">
-        <v>524</v>
+        <v>404</v>
       </c>
       <c r="C21" t="s">
         <v>13</v>
       </c>
       <c r="D21" t="s">
-        <v>569</v>
+        <v>449</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>570</v>
+        <v>450</v>
       </c>
       <c r="B22" t="s">
-        <v>524</v>
+        <v>404</v>
       </c>
       <c r="C22" t="s">
         <v>13</v>
       </c>
       <c r="D22" t="s">
-        <v>571</v>
+        <v>451</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>572</v>
+        <v>452</v>
       </c>
       <c r="B23" t="s">
         <v>13</v>
@@ -5198,35 +4260,35 @@
         <v>13</v>
       </c>
       <c r="D23" t="s">
-        <v>573</v>
+        <v>453</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>574</v>
+        <v>454</v>
       </c>
       <c r="B24" t="s">
-        <v>524</v>
+        <v>404</v>
       </c>
       <c r="C24" t="s">
         <v>13</v>
       </c>
       <c r="D24" t="s">
-        <v>575</v>
+        <v>455</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>576</v>
+        <v>456</v>
       </c>
       <c r="B25" t="s">
-        <v>577</v>
+        <v>457</v>
       </c>
       <c r="C25" t="s">
-        <v>578</v>
+        <v>458</v>
       </c>
       <c r="D25" t="s">
-        <v>579</v>
+        <v>459</v>
       </c>
     </row>
   </sheetData>

</xml_diff>